<commit_message>
Update Song values via web editor
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -498,7 +498,7 @@
         <v>ebouwbcw</v>
       </c>
       <c r="E6" t="str">
-        <v>Soman</v>
+        <v>aeroplane</v>
       </c>
     </row>
     <row r="7">
@@ -532,7 +532,7 @@
         <v>bouhfiqjqjd ne. r.  t</v>
       </c>
       <c r="E8" t="str">
-        <v>Sameer</v>
+        <v>jet</v>
       </c>
     </row>
   </sheetData>

</xml_diff>